<commit_message>
Update some codes for clarity
</commit_message>
<xml_diff>
--- a/RBC_IRF_matching/BP.xlsx
+++ b/RBC_IRF_matching/BP.xlsx
@@ -1,29 +1,48 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29029"/>
   <workbookPr defaultThemeVersion="124226"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://bankofenglandcouk-my.sharepoint.com/personal/david_murakami_bankofengland_co_uk/Documents/Documents/dynare/DSGE_mod/RBC_IRF_matching/"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="10" documentId="11_E6386AED79097EB3DF622AD6E9F6E93AEE5CB8F5" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{7084D09A-7187-407F-AF20-47035A410AA0}"/>
   <bookViews>
-    <workbookView xWindow="120" yWindow="120" windowWidth="28515" windowHeight="12585"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Tabelle1" sheetId="1" r:id="rId1"/>
     <sheet name="Tabelle2" sheetId="2" r:id="rId2"/>
     <sheet name="Tabelle3" sheetId="3" r:id="rId3"/>
   </sheets>
-  <calcPr calcId="145621"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
 <file path=xl/connections.xml><?xml version="1.0" encoding="utf-8"?>
-<connections xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <connection id="1" name="search" type="4" refreshedVersion="0" deleted="1" background="1">
+<connections xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr16="http://schemas.microsoft.com/office/spreadsheetml/2017/revision16" mc:Ignorable="xr16">
+  <connection id="1" xr16:uid="{00000000-0015-0000-FFFF-FFFF00000000}" name="search" type="4" refreshedVersion="0" deleted="1" background="1">
     <webPr xml="1" sourceData="1" url="http://api.stlouisfed.org/fred/series/search?search_text=PCND&amp;api_key=e2ddad77bf1066d5453b6e18f1f2958f&amp;search_type=full_text&amp;limit=100&amp;order_by=&amp;filter_variable=&amp;filter_value=&amp;sort_order=" htmlTables="1" htmlFormat="all"/>
   </connection>
-  <connection id="2" name="Verbindung" type="4" refreshedVersion="0" background="1">
+  <connection id="2" xr16:uid="{00000000-0015-0000-FFFF-FFFF01000000}" name="Verbindung" type="4" refreshedVersion="0" background="1">
     <webPr url="https://research.stlouisfed.org/fred2/data/Nipa Pop.txt" htmlTables="1" htmlFormat="all"/>
   </connection>
-  <connection id="3" name="Verbindung1" type="4" refreshedVersion="0" background="1">
+  <connection id="3" xr16:uid="{00000000-0015-0000-FFFF-FFFF02000000}" name="Verbindung1" type="4" refreshedVersion="0" background="1">
     <webPr url="https://research.stlouisfed.org/fred2/data/Nipa Pop.txt" htmlTables="1" htmlFormat="all"/>
   </connection>
 </connections>
@@ -962,7 +981,7 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="2">
     <numFmt numFmtId="164" formatCode="0.0"/>
     <numFmt numFmtId="165" formatCode="mm/dd/yyyy"/>
@@ -1019,13 +1038,16 @@
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
-    <cellStyle name="Standard" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
     </ext>
   </extLst>
 </styleSheet>
@@ -1076,9 +1098,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Larissa">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
   <a:themeElements>
-    <a:clrScheme name="Larissa">
+    <a:clrScheme name="Office 2007 - 2010">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -1116,7 +1138,7 @@
         <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Larissa">
+    <a:fontScheme name="Office 2007 - 2010">
       <a:majorFont>
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
@@ -1188,7 +1210,7 @@
         <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Larissa">
+    <a:fmtScheme name="Office 2007 - 2010">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -1361,24 +1383,24 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:O285"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="12" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="12" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="12" style="2"/>
     <col min="2" max="2" width="12" style="1"/>
     <col min="3" max="3" width="12" style="2"/>
     <col min="4" max="4" width="12" style="1"/>
-    <col min="5" max="5" width="12" style="2"/>
-    <col min="6" max="6" width="12" style="1"/>
-    <col min="7" max="7" width="12" style="2"/>
-    <col min="8" max="8" width="12" style="1"/>
-    <col min="9" max="9" width="12" style="2"/>
-    <col min="10" max="10" width="12" style="1"/>
-    <col min="11" max="11" width="12" style="2"/>
-    <col min="12" max="12" width="12" style="1"/>
-    <col min="13" max="13" width="12" style="2"/>
-    <col min="14" max="14" width="12" style="1"/>
+    <col min="5" max="5" width="57.7109375" style="2" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="23" style="1" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="33.42578125" style="2" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="23" style="1" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="52.140625" style="2" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="23" style="1" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="42.5703125" style="2" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="23" style="1" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="30.140625" style="2" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="23" style="1" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:15" x14ac:dyDescent="0.25">
@@ -14117,31 +14139,31 @@
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="A5" r:id="rId1"/>
-    <hyperlink ref="C5" r:id="rId2"/>
-    <hyperlink ref="E5" r:id="rId3"/>
-    <hyperlink ref="G5" r:id="rId4"/>
-    <hyperlink ref="I5" r:id="rId5"/>
-    <hyperlink ref="K5" r:id="rId6"/>
-    <hyperlink ref="M5" r:id="rId7"/>
+    <hyperlink ref="A5" r:id="rId1" xr:uid="{00000000-0004-0000-0000-000000000000}"/>
+    <hyperlink ref="C5" r:id="rId2" xr:uid="{00000000-0004-0000-0000-000001000000}"/>
+    <hyperlink ref="E5" r:id="rId3" xr:uid="{00000000-0004-0000-0000-000002000000}"/>
+    <hyperlink ref="G5" r:id="rId4" xr:uid="{00000000-0004-0000-0000-000003000000}"/>
+    <hyperlink ref="I5" r:id="rId5" xr:uid="{00000000-0004-0000-0000-000004000000}"/>
+    <hyperlink ref="K5" r:id="rId6" xr:uid="{00000000-0004-0000-0000-000005000000}"/>
+    <hyperlink ref="M5" r:id="rId7" xr:uid="{00000000-0004-0000-0000-000006000000}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData/>
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData/>
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>